<commit_message>
fixed part numbers and manufacturers
</commit_message>
<xml_diff>
--- a/library/transistors.xlsx
+++ b/library/transistors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0719BFAF-C805-4D4F-AE1B-3F0F2948E6DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5052B024-D0DE-4BC2-A8D5-BD92C103EC6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="nmos" sheetId="8" r:id="rId1"/>
@@ -1124,7 +1124,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5A36DDB-75CB-4526-8B7C-3E1D54E638B5}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.85546875" customWidth="1"/>
@@ -1202,12 +1202,12 @@
       <c r="F3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1225,7 +1225,7 @@
       <c r="F4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       <c r="F5" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -1317,21 +1317,21 @@
       <c r="F8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>75</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -1341,8 +1341,11 @@
         <v>24</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>74</v>
-      </c>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>